<commit_message>
fix: reject negative/zero amounts and raise on missing PDF
- validator.py: add amount > 0 check (closes #1, #2)
- pdf_parser.py: raise FileNotFoundError for missing files instead of silently returning (closes #3)
- qa/test_matrix.xlsx: updated — all 15 cases now pass
- qa/run_tests.py: test runner script

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/qa/test_matrix.xlsx
+++ b/qa/test_matrix.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -47,11 +47,6 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -65,7 +60,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -74,9 +69,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -765,7 +757,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>due_date=2026-06-28</t>
+          <t>due_date=2026-07-02</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -886,12 +878,12 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>No exception raised. Got: {'vendor': None, 'invoice_no': None, 'invoice_date': None, 'due_date': None, 'amount': None, 'currency': None, 'line_items': []}</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>Exception: PDF file not found: 'test_data/fake_invoice.pdf'</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -960,12 +952,12 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>{'valid': True, 'errors': []}</t>
-        </is>
-      </c>
-      <c r="F14" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>{'valid': False, 'errors': ['Amount must be greater than zero']}</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -997,12 +989,12 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>{'valid': True, 'errors': []}</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Fail</t>
+          <t>{'valid': False, 'errors': ['Amount must be greater than zero']}</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">

</xml_diff>